<commit_message>
session checkpoint: 2026-06-06 22:39
</commit_message>
<xml_diff>
--- a/tests/ExcelBaseTestData/formatting-testdata/FormattingSmorgasboard.xlsx
+++ b/tests/ExcelBaseTestData/formatting-testdata/FormattingSmorgasboard.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamleshn/workspace/joplin-univer/tests/ExcelBaseTestData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamleshn/workspace/joplin-univer/tests/ExcelBaseTestData/formatting-testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94E252E5-CA70-DF45-8207-93213A5A9021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E72B1C79-75F0-D149-B23A-67FB2824D6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13720" yWindow="660" windowWidth="15420" windowHeight="18980" xr2:uid="{8038F014-E0DA-9346-89F6-5C56764F8121}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{8038F014-E0DA-9346-89F6-5C56764F8121}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -237,24 +237,6 @@
         <sz val="11"/>
         <name val="Aptos"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <name val="Aptos"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <name val="Aptos"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <name val="Aptos"/>
-      </font>
       <numFmt numFmtId="19" formatCode="m/d/yy"/>
     </dxf>
     <dxf>
@@ -289,6 +271,24 @@
         <name val="Aptos"/>
       </font>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <name val="Aptos"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -334,16 +334,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33B3E454-1343-AF4D-8A75-918CC242F094}" name="ProjectTracker" displayName="ProjectTracker" ref="A1:G10" totalsRowCount="1" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33B3E454-1343-AF4D-8A75-918CC242F094}" name="ProjectTracker" displayName="ProjectTracker" ref="A1:G10" totalsRowCount="1" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
   <autoFilter ref="A1:G9" xr:uid="{33B3E454-1343-AF4D-8A75-918CC242F094}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{19393CFA-5FD9-594F-888E-0F27E7C6198A}" name="Project" totalsRowLabel="Totals" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{FD85AF8F-688B-7A40-B424-579D09690DB1}" name="Website" dataDxfId="14" totalsRowDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{9EE65B2E-ABE2-974F-B58B-E41E784F00A5}" name="Budget" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{812BB9FD-5302-E548-80E2-882BCF9F1210}" name="Spent" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{9AD95526-1178-B043-AD00-3E94D487EE04}" name="% Complete" totalsRowFunction="average" dataDxfId="8" totalsRowDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{9FCE0904-C3B3-8B4B-B6F2-D1D7A471D676}" name="Start Date" dataDxfId="6" totalsRowDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{0E005CD4-E11C-124F-BA4E-E09966294098}" name="Status" totalsRowFunction="count" dataDxfId="4" totalsRowDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{19393CFA-5FD9-594F-888E-0F27E7C6198A}" name="Project" totalsRowLabel="Totals" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{FD85AF8F-688B-7A40-B424-579D09690DB1}" name="Website" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9EE65B2E-ABE2-974F-B58B-E41E784F00A5}" name="Budget" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{812BB9FD-5302-E548-80E2-882BCF9F1210}" name="Spent" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{9AD95526-1178-B043-AD00-3E94D487EE04}" name="% Complete" totalsRowFunction="average" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{9FCE0904-C3B3-8B4B-B6F2-D1D7A471D676}" name="Start Date" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{0E005CD4-E11C-124F-BA4E-E09966294098}" name="Status" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -685,18 +685,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65803FC0-8692-194E-B237-756C39ACF19D}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1640625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="40" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -719,7 +710,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -742,7 +733,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -765,7 +756,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -788,7 +779,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -811,7 +802,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -834,7 +825,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -857,7 +848,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -880,7 +871,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -903,7 +894,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>

</xml_diff>